<commit_message>
Thêm tiền điều kiện cho case HC-V6-07
</commit_message>
<xml_diff>
--- a/docs/kịch bản kiểm tra hệ thống Trạng Nguyên_1.xlsx
+++ b/docs/kịch bản kiểm tra hệ thống Trạng Nguyên_1.xlsx
@@ -1,21 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30520"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E552B74D-88D0-4987-BA01-D977EEB0F896}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowWidth="28800" windowHeight="12180" firstSheet="1" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Kịch bản kiểm tra" sheetId="1" r:id="rId1"/>
     <sheet name="Webuser các V - Test case" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -32,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="223">
   <si>
     <t>STT</t>
   </si>
@@ -713,6 +709,9 @@
     <t>Luồng chuyển V6 → V5 (vào màn Thi hay)</t>
   </si>
   <si>
+    <t>Đã đăng nhập V6 và V5</t>
+  </si>
+  <si>
     <t>1. Click mục 'Thi Toán' trên menu V6 → chờ trang /thi-toan tải xong
 2. Click 1 tab kỳ thi (vd 'Thi VNMF (Lớp 1 - 2 - 3)')
 3. Cuộn xuống bảng chặng thi
@@ -867,57 +866,221 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <charset val="134"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF1F4E79"/>
       <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
     </font>
     <font>
       <i/>
       <sz val="12"/>
       <color rgb="FF595959"/>
       <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF595959"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FFFFFFFF"/>
       <name val="Times New Roman"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
-      <color rgb="FF595959"/>
-      <name val="Times New Roman"/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="40">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -926,136 +1089,239 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E79"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC55A11"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9E2F3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4D6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E79"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC55A11"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9E2F3"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFCE4D6"/>
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="20">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1110,166 +1376,535 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="176" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="12" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1318,7 +1953,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -1351,26 +1986,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -1403,23 +2021,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1561,354 +2162,349 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A3:K17"/>
-  <sheetFormatPr defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="1"/>
-    <col min="2" max="2" width="27.5703125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="36.7109375" style="3" customWidth="1"/>
-    <col min="4" max="4" width="32" style="3" customWidth="1"/>
-    <col min="5" max="5" width="32.85546875" style="3" customWidth="1"/>
-    <col min="6" max="6" width="34.7109375" style="3" customWidth="1"/>
-    <col min="7" max="7" width="29.42578125" style="3" customWidth="1"/>
-    <col min="8" max="8" width="35.85546875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="11.7109375" style="1" customWidth="1"/>
-    <col min="10" max="10" width="9.140625" style="3"/>
-    <col min="11" max="11" width="38.7109375" style="3" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="3"/>
+    <col min="1" max="1" width="9.14285714285714" style="17"/>
+    <col min="2" max="2" width="27.5714285714286" style="18" customWidth="1"/>
+    <col min="3" max="3" width="36.7142857142857" style="18" customWidth="1"/>
+    <col min="4" max="4" width="32" style="18" customWidth="1"/>
+    <col min="5" max="5" width="32.8571428571429" style="18" customWidth="1"/>
+    <col min="6" max="6" width="34.7142857142857" style="18" customWidth="1"/>
+    <col min="7" max="7" width="29.4285714285714" style="18" customWidth="1"/>
+    <col min="8" max="8" width="35.8571428571429" style="17" customWidth="1"/>
+    <col min="9" max="9" width="11.7142857142857" style="17" customWidth="1"/>
+    <col min="10" max="10" width="9.14285714285714" style="18"/>
+    <col min="11" max="11" width="38.7142857142857" style="18" customWidth="1"/>
+    <col min="12" max="16384" width="9.14285714285714" style="18"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:11" ht="19.5" customHeight="1">
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-    </row>
-    <row r="5" spans="1:11" ht="51" customHeight="1">
-      <c r="A5" s="4" t="s">
+    <row r="3" ht="19.5" customHeight="1" spans="1:11">
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+    </row>
+    <row r="5" ht="51" customHeight="1" spans="1:11">
+      <c r="A5" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="24" t="s">
+      <c r="G5" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="H5" s="30" t="s">
+      <c r="H5" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="I5" s="29" t="s">
+      <c r="I5" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="K5" s="10" t="s">
+      <c r="K5" s="29" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="61.5">
-      <c r="A6" s="11">
+    <row r="6" ht="63" spans="1:11">
+      <c r="A6" s="30">
         <v>1</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="D6" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="14" t="s">
+      <c r="E6" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="F6" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="G6" s="25" t="s">
+      <c r="G6" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="H6" s="26"/>
-      <c r="I6" s="11" t="s">
+      <c r="H6" s="36"/>
+      <c r="I6" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="K6" s="16" t="s">
+      <c r="K6" s="37" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="30.75">
-      <c r="A7" s="11">
+    <row r="7" ht="31.5" spans="1:11">
+      <c r="A7" s="30">
         <v>2</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="14" t="s">
+      <c r="F7" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="G7" s="26" t="s">
+      <c r="G7" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="26"/>
-      <c r="I7" s="11" t="s">
+      <c r="H7" s="36"/>
+      <c r="I7" s="30" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="73.5" customHeight="1">
-      <c r="A8" s="11">
+    <row r="8" ht="73.5" customHeight="1" spans="1:11">
+      <c r="A8" s="30">
         <v>3</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="D8" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="E8" s="17" t="s">
+      <c r="E8" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="F8" s="18" t="s">
+      <c r="F8" s="39" t="s">
         <v>27</v>
       </c>
-      <c r="G8" s="26" t="s">
+      <c r="G8" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="H8" s="31" t="s">
+      <c r="H8" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="I8" s="11" t="s">
+      <c r="I8" s="30" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="91.5">
-      <c r="A9" s="11">
+    <row r="9" ht="94.5" spans="1:11">
+      <c r="A9" s="30">
         <v>4</v>
       </c>
-      <c r="B9" s="48" t="s">
+      <c r="B9" s="41" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="27" t="s">
+      <c r="C9" s="42" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="28" t="s">
+      <c r="D9" s="43" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="27"/>
-      <c r="F9" s="28" t="s">
+      <c r="E9" s="42"/>
+      <c r="F9" s="43" t="s">
         <v>32</v>
       </c>
-      <c r="G9" s="26" t="s">
+      <c r="G9" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="H9" s="31" t="s">
+      <c r="H9" s="40" t="s">
         <v>33</v>
       </c>
-      <c r="I9" s="11" t="s">
+      <c r="I9" s="30" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="119.25" customHeight="1">
-      <c r="A10" s="11">
+    <row r="10" ht="119.25" customHeight="1" spans="1:11">
+      <c r="A10" s="30">
         <v>5</v>
       </c>
-      <c r="B10" s="49"/>
-      <c r="C10" s="17" t="s">
+      <c r="B10" s="44"/>
+      <c r="C10" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="D10" s="14" t="s">
+      <c r="D10" s="33" t="s">
         <v>35</v>
       </c>
-      <c r="E10" s="17"/>
-      <c r="F10" s="19" t="s">
+      <c r="E10" s="38"/>
+      <c r="F10" s="45" t="s">
         <v>36</v>
       </c>
-      <c r="G10" s="26" t="s">
+      <c r="G10" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="H10" s="31" t="s">
+      <c r="H10" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="I10" s="11" t="s">
+      <c r="I10" s="30" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="103.5" customHeight="1">
-      <c r="A11" s="11">
+    <row r="11" ht="103.5" customHeight="1" spans="1:11">
+      <c r="A11" s="30">
         <v>6</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="D11" s="14" t="s">
+      <c r="D11" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="E11" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="F11" s="19" t="s">
+      <c r="F11" s="45" t="s">
         <v>42</v>
       </c>
-      <c r="G11" s="26" t="s">
+      <c r="G11" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="H11" s="26" t="s">
+      <c r="H11" s="36" t="s">
         <v>43</v>
       </c>
-      <c r="I11" s="11" t="s">
+      <c r="I11" s="30" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:11">
-      <c r="I12" s="11"/>
+      <c r="I12" s="30"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="I13" s="11"/>
-    </row>
-    <row r="14" spans="1:11" ht="40.5" customHeight="1">
-      <c r="A14" s="11" t="s">
+      <c r="I13" s="30"/>
+    </row>
+    <row r="14" ht="40.5" customHeight="1" spans="1:11">
+      <c r="A14" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="G14" s="24" t="s">
+      <c r="G14" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="H14" s="30" t="s">
+      <c r="H14" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="I14" s="4"/>
-      <c r="K14" s="10" t="s">
+      <c r="I14" s="20"/>
+      <c r="K14" s="29" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="76.5" customHeight="1">
-      <c r="A15" s="11">
+    <row r="15" ht="76.5" customHeight="1" spans="1:11">
+      <c r="A15" s="30">
         <v>1</v>
       </c>
-      <c r="B15" s="20" t="s">
+      <c r="B15" s="46" t="s">
         <v>47</v>
       </c>
-      <c r="C15" s="21" t="s">
+      <c r="C15" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="D15" s="17" t="s">
+      <c r="D15" s="38" t="s">
         <v>49</v>
       </c>
-      <c r="E15" s="14" t="s">
+      <c r="E15" s="33" t="s">
         <v>50</v>
       </c>
-      <c r="F15" s="15" t="s">
+      <c r="F15" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="G15" s="26" t="s">
+      <c r="G15" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="H15" s="26"/>
-      <c r="I15" s="11" t="s">
+      <c r="H15" s="36"/>
+      <c r="I15" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="K15" s="16" t="s">
+      <c r="K15" s="37" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="35.25" customHeight="1">
-      <c r="A16" s="11">
+    <row r="16" ht="35.25" customHeight="1" spans="1:11">
+      <c r="A16" s="30">
         <v>2</v>
       </c>
-      <c r="B16" s="20" t="s">
+      <c r="B16" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="C16" s="22" t="s">
+      <c r="C16" s="48" t="s">
         <v>53</v>
       </c>
-      <c r="D16" s="17" t="s">
+      <c r="D16" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="E16" s="17" t="s">
+      <c r="E16" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="F16" s="23" t="s">
+      <c r="F16" s="49" t="s">
         <v>56</v>
       </c>
-      <c r="G16" s="26" t="s">
+      <c r="G16" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="H16" s="26"/>
-      <c r="I16" s="11" t="s">
+      <c r="H16" s="36"/>
+      <c r="I16" s="30" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="28.5" customHeight="1">
-      <c r="A17" s="11">
+    <row r="17" ht="28.5" customHeight="1" spans="1:9">
+      <c r="A17" s="30">
         <v>3</v>
       </c>
-      <c r="B17" s="20" t="s">
+      <c r="B17" s="46" t="s">
         <v>57</v>
       </c>
-      <c r="C17" s="22" t="s">
+      <c r="C17" s="48" t="s">
         <v>58</v>
       </c>
-      <c r="D17" s="17" t="s">
+      <c r="D17" s="38" t="s">
         <v>59</v>
       </c>
-      <c r="E17" s="17" t="s">
+      <c r="E17" s="38" t="s">
         <v>60</v>
       </c>
-      <c r="F17" s="14" t="s">
+      <c r="F17" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="G17" s="26" t="s">
+      <c r="G17" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="H17" s="26"/>
-      <c r="I17" s="11" t="s">
+      <c r="H17" s="36"/>
+      <c r="I17" s="30" t="s">
         <v>22</v>
       </c>
     </row>
@@ -1917,918 +2513,920 @@
     <mergeCell ref="B9:B10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{725696CC-6BC1-42CE-BFE2-CB0ABD653820}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:K33"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.85546875" customWidth="1"/>
-    <col min="2" max="2" width="12.85546875" customWidth="1"/>
-    <col min="3" max="3" width="32.28515625" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" customWidth="1"/>
-    <col min="5" max="5" width="27.42578125" customWidth="1"/>
-    <col min="6" max="6" width="70.42578125" customWidth="1"/>
-    <col min="7" max="7" width="55.85546875" customWidth="1"/>
-    <col min="8" max="8" width="33.7109375" customWidth="1"/>
-    <col min="9" max="9" width="47.42578125" customWidth="1"/>
-    <col min="10" max="10" width="50.7109375" customWidth="1"/>
-    <col min="11" max="11" width="48.42578125" customWidth="1"/>
+    <col min="1" max="1" width="16.8571428571429" customWidth="1"/>
+    <col min="2" max="2" width="12.8571428571429" customWidth="1"/>
+    <col min="3" max="3" width="32.2857142857143" customWidth="1"/>
+    <col min="4" max="4" width="11.7142857142857" customWidth="1"/>
+    <col min="5" max="5" width="27.4285714285714" customWidth="1"/>
+    <col min="6" max="6" width="70.4285714285714" customWidth="1"/>
+    <col min="7" max="7" width="55.8571428571429" customWidth="1"/>
+    <col min="8" max="8" width="33.7142857142857" customWidth="1"/>
+    <col min="9" max="9" width="47.4285714285714" customWidth="1"/>
+    <col min="10" max="10" width="50.7142857142857" customWidth="1"/>
+    <col min="11" max="11" width="48.4285714285714" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="34" customFormat="1" ht="36" customHeight="1">
-      <c r="A1" s="43" t="s">
+    <row r="1" s="1" customFormat="1" ht="36" customHeight="1" spans="1:11">
+      <c r="A1" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
-    </row>
-    <row r="2" spans="1:11" ht="24" customHeight="1">
-      <c r="A2" s="33" t="s">
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
+    </row>
+    <row r="2" ht="24" customHeight="1" spans="1:11">
+      <c r="A2" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="32"/>
-    </row>
-    <row r="3" spans="1:11" ht="24" customHeight="1">
-      <c r="A3" s="33" t="s">
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
+    </row>
+    <row r="3" ht="24" customHeight="1" spans="1:11">
+      <c r="A3" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="B3" s="32"/>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32"/>
-      <c r="I3" s="32"/>
-      <c r="J3" s="32"/>
-      <c r="K3" s="32"/>
-    </row>
-    <row r="4" spans="1:11" ht="24" customHeight="1">
-      <c r="A4" s="33" t="s">
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
+    </row>
+    <row r="4" ht="24" customHeight="1" spans="1:11">
+      <c r="A4" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B4" s="32"/>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="32"/>
-      <c r="F4" s="32"/>
-      <c r="G4" s="32"/>
-      <c r="H4" s="32"/>
-      <c r="I4" s="32"/>
-      <c r="J4" s="32"/>
-      <c r="K4" s="32"/>
-    </row>
-    <row r="5" spans="1:11" ht="24" customHeight="1">
-      <c r="A5" s="33" t="s">
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+    </row>
+    <row r="5" ht="24" customHeight="1" spans="1:11">
+      <c r="A5" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="B5" s="32"/>
-      <c r="C5" s="32"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="32"/>
-      <c r="G5" s="32"/>
-      <c r="H5" s="32"/>
-      <c r="I5" s="32"/>
-      <c r="J5" s="32"/>
-      <c r="K5" s="32"/>
-    </row>
-    <row r="6" spans="1:11" ht="24" customHeight="1">
-      <c r="A6" s="33" t="s">
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+    </row>
+    <row r="6" ht="24" customHeight="1" spans="1:11">
+      <c r="A6" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B6" s="32"/>
-      <c r="C6" s="32"/>
-      <c r="D6" s="32"/>
-      <c r="E6" s="32"/>
-      <c r="F6" s="32"/>
-      <c r="G6" s="32"/>
-      <c r="H6" s="32"/>
-      <c r="I6" s="32"/>
-      <c r="J6" s="32"/>
-      <c r="K6" s="32"/>
-    </row>
-    <row r="7" spans="1:11" ht="24" customHeight="1">
-      <c r="A7" s="33" t="s">
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+    </row>
+    <row r="7" ht="24" customHeight="1" spans="1:11">
+      <c r="A7" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="B7" s="32"/>
-      <c r="C7" s="32"/>
-      <c r="D7" s="32"/>
-      <c r="E7" s="32"/>
-      <c r="F7" s="32"/>
-      <c r="G7" s="32"/>
-      <c r="H7" s="32"/>
-      <c r="I7" s="32"/>
-      <c r="J7" s="32"/>
-      <c r="K7" s="32"/>
-    </row>
-    <row r="8" spans="1:11" ht="24" customHeight="1">
-      <c r="A8" s="50" t="s">
+      <c r="B7" s="7"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+    </row>
+    <row r="8" ht="24" customHeight="1" spans="1:11">
+      <c r="A8" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="B8" s="32"/>
-      <c r="C8" s="32"/>
-      <c r="D8" s="32"/>
-      <c r="E8" s="32"/>
-      <c r="F8" s="32"/>
-      <c r="G8" s="32"/>
-      <c r="H8" s="32"/>
-      <c r="I8" s="32"/>
-      <c r="J8" s="32"/>
-      <c r="K8" s="32"/>
-    </row>
-    <row r="9" spans="1:11" ht="24" customHeight="1">
-      <c r="A9" s="50" t="s">
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+    </row>
+    <row r="9" ht="24" customHeight="1" spans="1:11">
+      <c r="A9" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="B9" s="32"/>
-      <c r="C9" s="32"/>
-      <c r="D9" s="32"/>
-      <c r="E9" s="32"/>
-      <c r="F9" s="32"/>
-      <c r="G9" s="32"/>
-      <c r="H9" s="32"/>
-      <c r="I9" s="32"/>
-      <c r="J9" s="32"/>
-      <c r="K9" s="32"/>
-    </row>
-    <row r="10" spans="1:11" ht="15.75">
-      <c r="A10" s="32"/>
-      <c r="B10" s="32"/>
-      <c r="C10" s="32"/>
-      <c r="D10" s="32"/>
-      <c r="E10" s="32"/>
-      <c r="F10" s="32"/>
-      <c r="G10" s="32"/>
-      <c r="H10" s="32"/>
-      <c r="I10" s="32"/>
-      <c r="J10" s="32"/>
-      <c r="K10" s="32"/>
-    </row>
-    <row r="11" spans="1:11" s="37" customFormat="1" ht="36.75" customHeight="1">
-      <c r="A11" s="35" t="s">
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+    </row>
+    <row r="10" ht="15.75" spans="1:11">
+      <c r="A10" s="7"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+    </row>
+    <row r="11" s="2" customFormat="1" ht="36.75" customHeight="1" spans="1:11">
+      <c r="A11" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="B11" s="35" t="s">
+      <c r="B11" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C11" s="35" t="s">
+      <c r="C11" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="D11" s="35" t="s">
+      <c r="D11" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="E11" s="35" t="s">
+      <c r="E11" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="F11" s="35" t="s">
+      <c r="F11" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="G11" s="35" t="s">
+      <c r="G11" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="H11" s="35" t="s">
+      <c r="H11" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="I11" s="35" t="s">
+      <c r="I11" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="J11" s="36" t="s">
+      <c r="J11" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="K11" s="35" t="s">
+      <c r="K11" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="12" spans="1:11" s="34" customFormat="1" ht="21" customHeight="1">
-      <c r="A12" s="45" t="s">
+    <row r="12" s="1" customFormat="1" ht="21" customHeight="1" spans="1:11">
+      <c r="A12" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="B12" s="46"/>
-      <c r="C12" s="46"/>
-      <c r="D12" s="46"/>
-      <c r="E12" s="46"/>
-      <c r="F12" s="46"/>
-      <c r="G12" s="46"/>
-      <c r="H12" s="46"/>
-      <c r="I12" s="46"/>
-      <c r="J12" s="46"/>
-      <c r="K12" s="47"/>
-    </row>
-    <row r="13" spans="1:11" s="42" customFormat="1" ht="137.25" customHeight="1">
-      <c r="A13" s="38" t="s">
+      <c r="B12" s="12"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="12"/>
+      <c r="J12" s="12"/>
+      <c r="K12" s="13"/>
+    </row>
+    <row r="13" s="3" customFormat="1" ht="137.25" customHeight="1" spans="1:11">
+      <c r="A13" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="B13" s="39" t="s">
+      <c r="B13" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="C13" s="39" t="s">
+      <c r="C13" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="D13" s="39" t="s">
+      <c r="D13" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="E13" s="39" t="s">
+      <c r="E13" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="F13" s="39" t="s">
+      <c r="F13" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="G13" s="40" t="s">
+      <c r="G13" s="50" t="s">
         <v>89</v>
       </c>
-      <c r="H13" s="40" t="s">
+      <c r="H13" s="50" t="s">
         <v>90</v>
       </c>
-      <c r="I13" s="40" t="s">
+      <c r="I13" s="50" t="s">
         <v>91</v>
       </c>
-      <c r="J13" s="41" t="s">
+      <c r="J13" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="K13" s="39" t="s">
+      <c r="K13" s="15" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="14" spans="1:11" s="42" customFormat="1" ht="137.25" customHeight="1">
-      <c r="A14" s="38" t="s">
+    <row r="14" s="3" customFormat="1" ht="137.25" customHeight="1" spans="1:11">
+      <c r="A14" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="B14" s="39" t="s">
+      <c r="B14" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="C14" s="39" t="s">
+      <c r="C14" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="D14" s="39" t="s">
+      <c r="D14" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="E14" s="39" t="s">
+      <c r="E14" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="F14" s="39" t="s">
+      <c r="F14" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="G14" s="40" t="s">
+      <c r="G14" s="50" t="s">
         <v>98</v>
       </c>
-      <c r="H14" s="40" t="s">
+      <c r="H14" s="50" t="s">
         <v>99</v>
       </c>
-      <c r="I14" s="40" t="s">
+      <c r="I14" s="50" t="s">
         <v>100</v>
       </c>
-      <c r="J14" s="41" t="s">
+      <c r="J14" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="K14" s="39" t="s">
+      <c r="K14" s="15" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="15" spans="1:11" s="42" customFormat="1" ht="137.25" customHeight="1">
-      <c r="A15" s="38" t="s">
+    <row r="15" s="3" customFormat="1" ht="137.25" customHeight="1" spans="1:11">
+      <c r="A15" s="14" t="s">
         <v>103</v>
       </c>
-      <c r="B15" s="39" t="s">
+      <c r="B15" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="C15" s="39" t="s">
+      <c r="C15" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="D15" s="39" t="s">
+      <c r="D15" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="E15" s="39" t="s">
+      <c r="E15" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="F15" s="39" t="s">
+      <c r="F15" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="G15" s="40" t="s">
+      <c r="G15" s="50" t="s">
         <v>107</v>
       </c>
-      <c r="H15" s="40" t="s">
+      <c r="H15" s="50" t="s">
         <v>99</v>
       </c>
-      <c r="I15" s="40" t="s">
+      <c r="I15" s="50" t="s">
         <v>108</v>
       </c>
-      <c r="J15" s="41" t="s">
+      <c r="J15" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="K15" s="39" t="s">
+      <c r="K15" s="15" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="16" spans="1:11" s="42" customFormat="1" ht="92.25" customHeight="1">
-      <c r="A16" s="38" t="s">
+    <row r="16" s="3" customFormat="1" ht="92.25" customHeight="1" spans="1:11">
+      <c r="A16" s="14" t="s">
         <v>110</v>
       </c>
-      <c r="B16" s="39" t="s">
+      <c r="B16" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="C16" s="39" t="s">
+      <c r="C16" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="D16" s="39" t="s">
+      <c r="D16" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="E16" s="39" t="s">
+      <c r="E16" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="F16" s="39" t="s">
+      <c r="F16" s="15" t="s">
         <v>113</v>
       </c>
-      <c r="G16" s="40" t="s">
+      <c r="G16" s="50" t="s">
         <v>114</v>
       </c>
-      <c r="H16" s="40" t="s">
+      <c r="H16" s="50" t="s">
         <v>99</v>
       </c>
-      <c r="I16" s="40" t="s">
+      <c r="I16" s="50" t="s">
         <v>115</v>
       </c>
-      <c r="J16" s="41" t="s">
+      <c r="J16" s="16" t="s">
         <v>116</v>
       </c>
-      <c r="K16" s="39" t="s">
+      <c r="K16" s="15" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="17" spans="1:11" s="42" customFormat="1" ht="67.5" customHeight="1">
-      <c r="A17" s="38" t="s">
+    <row r="17" s="3" customFormat="1" ht="67.5" customHeight="1" spans="1:11">
+      <c r="A17" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="B17" s="39" t="s">
+      <c r="B17" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="C17" s="39" t="s">
+      <c r="C17" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="D17" s="39" t="s">
+      <c r="D17" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="E17" s="39" t="s">
+      <c r="E17" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="F17" s="39" t="s">
+      <c r="F17" s="15" t="s">
         <v>121</v>
       </c>
-      <c r="G17" s="40" t="s">
+      <c r="G17" s="50" t="s">
         <v>122</v>
       </c>
-      <c r="H17" s="40" t="s">
+      <c r="H17" s="50" t="s">
         <v>99</v>
       </c>
-      <c r="I17" s="40" t="s">
+      <c r="I17" s="50" t="s">
         <v>123</v>
       </c>
-      <c r="J17" s="41" t="s">
+      <c r="J17" s="16" t="s">
         <v>124</v>
       </c>
-      <c r="K17" s="39" t="s">
+      <c r="K17" s="15" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="18" spans="1:11" s="42" customFormat="1" ht="68.25" customHeight="1">
-      <c r="A18" s="38" t="s">
+    <row r="18" s="3" customFormat="1" ht="68.25" customHeight="1" spans="1:11">
+      <c r="A18" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="B18" s="39" t="s">
+      <c r="B18" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="C18" s="39" t="s">
+      <c r="C18" s="15" t="s">
         <v>127</v>
       </c>
-      <c r="D18" s="39" t="s">
+      <c r="D18" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="E18" s="39" t="s">
+      <c r="E18" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="F18" s="39" t="s">
+      <c r="F18" s="15" t="s">
         <v>128</v>
       </c>
-      <c r="G18" s="40" t="s">
+      <c r="G18" s="50" t="s">
         <v>129</v>
       </c>
-      <c r="H18" s="40" t="s">
+      <c r="H18" s="50" t="s">
         <v>99</v>
       </c>
-      <c r="I18" s="40" t="s">
+      <c r="I18" s="50" t="s">
         <v>130</v>
       </c>
-      <c r="J18" s="41" t="s">
+      <c r="J18" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="K18" s="39" t="s">
+      <c r="K18" s="15" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="19" spans="1:11" s="42" customFormat="1" ht="72" customHeight="1">
-      <c r="A19" s="38" t="s">
+    <row r="19" s="3" customFormat="1" ht="72" customHeight="1" spans="1:11">
+      <c r="A19" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="B19" s="39" t="s">
+      <c r="B19" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="C19" s="39" t="s">
+      <c r="C19" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="D19" s="39" t="s">
+      <c r="D19" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="E19" s="39" t="s">
+      <c r="E19" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="F19" s="39" t="s">
+      <c r="F19" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="G19" s="40" t="s">
+      <c r="G19" s="50" t="s">
         <v>136</v>
       </c>
-      <c r="H19" s="40" t="s">
+      <c r="H19" s="50" t="s">
         <v>137</v>
       </c>
-      <c r="I19" s="40" t="s">
+      <c r="I19" s="50" t="s">
         <v>138</v>
       </c>
-      <c r="J19" s="41" t="s">
+      <c r="J19" s="16" t="s">
         <v>139</v>
       </c>
-      <c r="K19" s="39" t="s">
+      <c r="K19" s="15" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="20" spans="1:11" s="34" customFormat="1" ht="21.75" customHeight="1">
-      <c r="A20" s="45" t="s">
+    <row r="20" s="1" customFormat="1" ht="21.75" customHeight="1" spans="1:11">
+      <c r="A20" s="11" t="s">
         <v>141</v>
       </c>
-      <c r="B20" s="46"/>
-      <c r="C20" s="46"/>
-      <c r="D20" s="46"/>
-      <c r="E20" s="46"/>
-      <c r="F20" s="46"/>
-      <c r="G20" s="46"/>
-      <c r="H20" s="46"/>
-      <c r="I20" s="46"/>
-      <c r="J20" s="46"/>
-      <c r="K20" s="47"/>
-    </row>
-    <row r="21" spans="1:11" s="42" customFormat="1" ht="107.25">
-      <c r="A21" s="38" t="s">
+      <c r="B20" s="12"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="12"/>
+      <c r="I20" s="12"/>
+      <c r="J20" s="12"/>
+      <c r="K20" s="13"/>
+    </row>
+    <row r="21" s="3" customFormat="1" ht="110.25" spans="1:11">
+      <c r="A21" s="14" t="s">
         <v>142</v>
       </c>
-      <c r="B21" s="39" t="s">
+      <c r="B21" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="C21" s="39" t="s">
+      <c r="C21" s="15" t="s">
         <v>144</v>
       </c>
-      <c r="D21" s="39" t="s">
+      <c r="D21" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="E21" s="39" t="s">
+      <c r="E21" s="15" t="s">
         <v>145</v>
       </c>
-      <c r="F21" s="39" t="s">
+      <c r="F21" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="G21" s="40" t="s">
+      <c r="G21" s="50" t="s">
         <v>147</v>
       </c>
-      <c r="H21" s="40" t="s">
+      <c r="H21" s="50" t="s">
         <v>148</v>
       </c>
-      <c r="I21" s="40" t="s">
+      <c r="I21" s="50" t="s">
         <v>149</v>
       </c>
-      <c r="J21" s="41" t="s">
+      <c r="J21" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="K21" s="39" t="s">
+      <c r="K21" s="15" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="22" spans="1:11" s="42" customFormat="1" ht="137.25">
-      <c r="A22" s="38" t="s">
+    <row r="22" s="3" customFormat="1" ht="110.25" spans="1:11">
+      <c r="A22" s="14" t="s">
         <v>152</v>
       </c>
-      <c r="B22" s="39" t="s">
+      <c r="B22" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="C22" s="39" t="s">
+      <c r="C22" s="15" t="s">
         <v>153</v>
       </c>
-      <c r="D22" s="39" t="s">
+      <c r="D22" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="E22" s="39" t="s">
+      <c r="E22" s="15" t="s">
         <v>154</v>
       </c>
-      <c r="F22" s="39" t="s">
+      <c r="F22" s="15" t="s">
         <v>155</v>
       </c>
-      <c r="G22" s="40" t="s">
+      <c r="G22" s="50" t="s">
         <v>114</v>
       </c>
-      <c r="H22" s="40" t="s">
+      <c r="H22" s="50" t="s">
         <v>99</v>
       </c>
-      <c r="I22" s="40" t="s">
+      <c r="I22" s="50" t="s">
         <v>115</v>
       </c>
-      <c r="J22" s="41" t="s">
+      <c r="J22" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="K22" s="39" t="s">
+      <c r="K22" s="15" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="23" spans="1:11" s="42" customFormat="1" ht="91.5">
-      <c r="A23" s="38" t="s">
+    <row r="23" s="3" customFormat="1" ht="94.5" spans="1:11">
+      <c r="A23" s="14" t="s">
         <v>158</v>
       </c>
-      <c r="B23" s="39" t="s">
+      <c r="B23" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="C23" s="39" t="s">
+      <c r="C23" s="15" t="s">
         <v>159</v>
       </c>
-      <c r="D23" s="39" t="s">
+      <c r="D23" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="E23" s="39" t="s">
+      <c r="E23" s="15" t="s">
         <v>160</v>
       </c>
-      <c r="F23" s="39" t="s">
+      <c r="F23" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="G23" s="40" t="s">
+      <c r="G23" s="50" t="s">
         <v>162</v>
       </c>
-      <c r="H23" s="40" t="s">
+      <c r="H23" s="50" t="s">
         <v>99</v>
       </c>
-      <c r="I23" s="40" t="s">
+      <c r="I23" s="50" t="s">
         <v>163</v>
       </c>
-      <c r="J23" s="41" t="s">
+      <c r="J23" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="K23" s="39" t="s">
+      <c r="K23" s="15" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="24" spans="1:11" s="42" customFormat="1" ht="107.25">
-      <c r="A24" s="38" t="s">
+    <row r="24" s="3" customFormat="1" ht="110.25" spans="1:11">
+      <c r="A24" s="14" t="s">
         <v>164</v>
       </c>
-      <c r="B24" s="39" t="s">
+      <c r="B24" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="C24" s="39" t="s">
+      <c r="C24" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="D24" s="39" t="s">
+      <c r="D24" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="E24" s="39" t="s">
+      <c r="E24" s="15" t="s">
         <v>160</v>
       </c>
-      <c r="F24" s="39" t="s">
+      <c r="F24" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="G24" s="40" t="s">
+      <c r="G24" s="50" t="s">
         <v>167</v>
       </c>
-      <c r="H24" s="40" t="s">
+      <c r="H24" s="50" t="s">
         <v>99</v>
       </c>
-      <c r="I24" s="40" t="s">
+      <c r="I24" s="50" t="s">
         <v>168</v>
       </c>
-      <c r="J24" s="41" t="s">
+      <c r="J24" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="K24" s="39" t="s">
+      <c r="K24" s="15" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="25" spans="1:11" s="42" customFormat="1" ht="121.5">
-      <c r="A25" s="38" t="s">
+    <row r="25" s="3" customFormat="1" ht="126" spans="1:11">
+      <c r="A25" s="14" t="s">
         <v>169</v>
       </c>
-      <c r="B25" s="39" t="s">
+      <c r="B25" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="C25" s="39" t="s">
+      <c r="C25" s="15" t="s">
         <v>170</v>
       </c>
-      <c r="D25" s="39" t="s">
+      <c r="D25" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="E25" s="39" t="s">
+      <c r="E25" s="15" t="s">
         <v>171</v>
       </c>
-      <c r="F25" s="39" t="s">
+      <c r="F25" s="15" t="s">
         <v>172</v>
       </c>
-      <c r="G25" s="40" t="s">
+      <c r="G25" s="50" t="s">
         <v>107</v>
       </c>
-      <c r="H25" s="40" t="s">
+      <c r="H25" s="50" t="s">
         <v>99</v>
       </c>
-      <c r="I25" s="40" t="s">
+      <c r="I25" s="50" t="s">
         <v>108</v>
       </c>
-      <c r="J25" s="41" t="s">
+      <c r="J25" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="K25" s="39" t="s">
+      <c r="K25" s="15" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="26" spans="1:11" s="42" customFormat="1" ht="61.5">
-      <c r="A26" s="38" t="s">
+    <row r="26" s="3" customFormat="1" ht="63" spans="1:11">
+      <c r="A26" s="14" t="s">
         <v>174</v>
       </c>
-      <c r="B26" s="39" t="s">
+      <c r="B26" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="C26" s="39" t="s">
+      <c r="C26" s="15" t="s">
         <v>175</v>
       </c>
-      <c r="D26" s="39" t="s">
+      <c r="D26" s="15" t="s">
         <v>176</v>
       </c>
-      <c r="E26" s="39" t="s">
+      <c r="E26" s="15" t="s">
         <v>171</v>
       </c>
-      <c r="F26" s="39" t="s">
+      <c r="F26" s="15" t="s">
         <v>177</v>
       </c>
-      <c r="G26" s="40" t="s">
+      <c r="G26" s="50" t="s">
         <v>178</v>
       </c>
-      <c r="H26" s="40" t="s">
+      <c r="H26" s="50" t="s">
         <v>99</v>
       </c>
-      <c r="I26" s="40" t="s">
+      <c r="I26" s="50" t="s">
         <v>179</v>
       </c>
-      <c r="J26" s="41" t="s">
+      <c r="J26" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="K26" s="39" t="s">
+      <c r="K26" s="15" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="27" spans="1:11" s="42" customFormat="1" ht="91.5">
-      <c r="A27" s="38" t="s">
+    <row r="27" s="3" customFormat="1" ht="94.5" spans="1:11">
+      <c r="A27" s="14" t="s">
         <v>182</v>
       </c>
-      <c r="B27" s="39" t="s">
+      <c r="B27" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="C27" s="39" t="s">
+      <c r="C27" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="D27" s="39" t="s">
+      <c r="D27" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="E27" s="39" t="s">
+      <c r="E27" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="F27" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="G27" s="50" t="s">
+        <v>186</v>
+      </c>
+      <c r="H27" s="50" t="s">
+        <v>99</v>
+      </c>
+      <c r="I27" s="50" t="s">
+        <v>187</v>
+      </c>
+      <c r="J27" s="16" t="s">
+        <v>188</v>
+      </c>
+      <c r="K27" s="15" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="28" s="3" customFormat="1" ht="47.25" spans="1:11">
+      <c r="A28" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="C28" s="15" t="s">
+        <v>191</v>
+      </c>
+      <c r="D28" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="E28" s="15" t="s">
         <v>171</v>
       </c>
-      <c r="F27" s="39" t="s">
-        <v>184</v>
-      </c>
-      <c r="G27" s="40" t="s">
-        <v>185</v>
-      </c>
-      <c r="H27" s="40" t="s">
+      <c r="F28" s="15" t="s">
+        <v>192</v>
+      </c>
+      <c r="G28" s="50" t="s">
+        <v>193</v>
+      </c>
+      <c r="H28" s="50" t="s">
         <v>99</v>
       </c>
-      <c r="I27" s="40" t="s">
-        <v>186</v>
-      </c>
-      <c r="J27" s="41" t="s">
-        <v>187</v>
-      </c>
-      <c r="K27" s="39" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" s="42" customFormat="1" ht="45.75">
-      <c r="A28" s="38" t="s">
-        <v>189</v>
-      </c>
-      <c r="B28" s="39" t="s">
+      <c r="I28" s="50" t="s">
+        <v>130</v>
+      </c>
+      <c r="J28" s="16" t="s">
+        <v>194</v>
+      </c>
+      <c r="K28" s="15" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="29" s="3" customFormat="1" ht="31.5" spans="1:11">
+      <c r="A29" s="14" t="s">
+        <v>196</v>
+      </c>
+      <c r="B29" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="C28" s="39" t="s">
-        <v>190</v>
-      </c>
-      <c r="D28" s="39" t="s">
+      <c r="C29" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="D29" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="E28" s="39" t="s">
+      <c r="E29" s="15" t="s">
         <v>171</v>
       </c>
-      <c r="F28" s="39" t="s">
-        <v>191</v>
-      </c>
-      <c r="G28" s="40" t="s">
-        <v>192</v>
-      </c>
-      <c r="H28" s="40" t="s">
+      <c r="F29" s="15" t="s">
+        <v>197</v>
+      </c>
+      <c r="G29" s="50" t="s">
+        <v>198</v>
+      </c>
+      <c r="H29" s="50" t="s">
+        <v>137</v>
+      </c>
+      <c r="I29" s="50" t="s">
+        <v>138</v>
+      </c>
+      <c r="J29" s="16" t="s">
+        <v>199</v>
+      </c>
+      <c r="K29" s="15" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="30" s="1" customFormat="1" ht="21.75" customHeight="1" spans="1:11">
+      <c r="A30" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="B30" s="12"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="12"/>
+      <c r="H30" s="12"/>
+      <c r="I30" s="12"/>
+      <c r="J30" s="12"/>
+      <c r="K30" s="13"/>
+    </row>
+    <row r="31" s="3" customFormat="1" ht="78.75" spans="1:11">
+      <c r="A31" s="14" t="s">
+        <v>202</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>203</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>204</v>
+      </c>
+      <c r="D31" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="E31" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="F31" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="G31" s="50" t="s">
+        <v>207</v>
+      </c>
+      <c r="H31" s="50" t="s">
         <v>99</v>
       </c>
-      <c r="I28" s="40" t="s">
+      <c r="I31" s="50" t="s">
+        <v>208</v>
+      </c>
+      <c r="J31" s="16" t="s">
+        <v>209</v>
+      </c>
+      <c r="K31" s="15" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="32" s="3" customFormat="1" ht="63" spans="1:11">
+      <c r="A32" s="14" t="s">
+        <v>211</v>
+      </c>
+      <c r="B32" s="15" t="s">
+        <v>203</v>
+      </c>
+      <c r="C32" s="15" t="s">
+        <v>212</v>
+      </c>
+      <c r="D32" s="15" t="s">
+        <v>213</v>
+      </c>
+      <c r="E32" s="15" t="s">
+        <v>214</v>
+      </c>
+      <c r="F32" s="15" t="s">
+        <v>215</v>
+      </c>
+      <c r="G32" s="50" t="s">
+        <v>216</v>
+      </c>
+      <c r="H32" s="50" t="s">
+        <v>99</v>
+      </c>
+      <c r="I32" s="50" t="s">
+        <v>217</v>
+      </c>
+      <c r="J32" s="16" t="s">
+        <v>218</v>
+      </c>
+      <c r="K32" s="15" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="33" s="3" customFormat="1" ht="47.25" spans="1:11">
+      <c r="A33" s="14" t="s">
+        <v>219</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>203</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>220</v>
+      </c>
+      <c r="D33" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="E33" s="15" t="s">
+        <v>214</v>
+      </c>
+      <c r="F33" s="15" t="s">
+        <v>221</v>
+      </c>
+      <c r="G33" s="50" t="s">
+        <v>222</v>
+      </c>
+      <c r="H33" s="50" t="s">
+        <v>99</v>
+      </c>
+      <c r="I33" s="50" t="s">
         <v>130</v>
       </c>
-      <c r="J28" s="41" t="s">
-        <v>193</v>
-      </c>
-      <c r="K28" s="39" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" s="42" customFormat="1" ht="45.75">
-      <c r="A29" s="38" t="s">
+      <c r="J33" s="16" t="s">
+        <v>131</v>
+      </c>
+      <c r="K33" s="15" t="s">
         <v>195</v>
-      </c>
-      <c r="B29" s="39" t="s">
-        <v>143</v>
-      </c>
-      <c r="C29" s="39" t="s">
-        <v>134</v>
-      </c>
-      <c r="D29" s="39" t="s">
-        <v>86</v>
-      </c>
-      <c r="E29" s="39" t="s">
-        <v>171</v>
-      </c>
-      <c r="F29" s="39" t="s">
-        <v>196</v>
-      </c>
-      <c r="G29" s="40" t="s">
-        <v>197</v>
-      </c>
-      <c r="H29" s="40" t="s">
-        <v>137</v>
-      </c>
-      <c r="I29" s="40" t="s">
-        <v>138</v>
-      </c>
-      <c r="J29" s="41" t="s">
-        <v>198</v>
-      </c>
-      <c r="K29" s="39" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" s="34" customFormat="1" ht="21.75" customHeight="1">
-      <c r="A30" s="45" t="s">
-        <v>200</v>
-      </c>
-      <c r="B30" s="46"/>
-      <c r="C30" s="46"/>
-      <c r="D30" s="46"/>
-      <c r="E30" s="46"/>
-      <c r="F30" s="46"/>
-      <c r="G30" s="46"/>
-      <c r="H30" s="46"/>
-      <c r="I30" s="46"/>
-      <c r="J30" s="46"/>
-      <c r="K30" s="47"/>
-    </row>
-    <row r="31" spans="1:11" s="42" customFormat="1" ht="76.5">
-      <c r="A31" s="38" t="s">
-        <v>201</v>
-      </c>
-      <c r="B31" s="39" t="s">
-        <v>202</v>
-      </c>
-      <c r="C31" s="39" t="s">
-        <v>203</v>
-      </c>
-      <c r="D31" s="39" t="s">
-        <v>176</v>
-      </c>
-      <c r="E31" s="39" t="s">
-        <v>204</v>
-      </c>
-      <c r="F31" s="39" t="s">
-        <v>205</v>
-      </c>
-      <c r="G31" s="40" t="s">
-        <v>206</v>
-      </c>
-      <c r="H31" s="40" t="s">
-        <v>99</v>
-      </c>
-      <c r="I31" s="40" t="s">
-        <v>207</v>
-      </c>
-      <c r="J31" s="41" t="s">
-        <v>208</v>
-      </c>
-      <c r="K31" s="39" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" s="42" customFormat="1" ht="61.5">
-      <c r="A32" s="38" t="s">
-        <v>210</v>
-      </c>
-      <c r="B32" s="39" t="s">
-        <v>202</v>
-      </c>
-      <c r="C32" s="39" t="s">
-        <v>211</v>
-      </c>
-      <c r="D32" s="39" t="s">
-        <v>212</v>
-      </c>
-      <c r="E32" s="39" t="s">
-        <v>213</v>
-      </c>
-      <c r="F32" s="39" t="s">
-        <v>214</v>
-      </c>
-      <c r="G32" s="40" t="s">
-        <v>215</v>
-      </c>
-      <c r="H32" s="40" t="s">
-        <v>99</v>
-      </c>
-      <c r="I32" s="40" t="s">
-        <v>216</v>
-      </c>
-      <c r="J32" s="41" t="s">
-        <v>217</v>
-      </c>
-      <c r="K32" s="39" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" s="42" customFormat="1" ht="45.75">
-      <c r="A33" s="38" t="s">
-        <v>218</v>
-      </c>
-      <c r="B33" s="39" t="s">
-        <v>202</v>
-      </c>
-      <c r="C33" s="39" t="s">
-        <v>219</v>
-      </c>
-      <c r="D33" s="39" t="s">
-        <v>86</v>
-      </c>
-      <c r="E33" s="39" t="s">
-        <v>213</v>
-      </c>
-      <c r="F33" s="39" t="s">
-        <v>220</v>
-      </c>
-      <c r="G33" s="40" t="s">
-        <v>221</v>
-      </c>
-      <c r="H33" s="40" t="s">
-        <v>99</v>
-      </c>
-      <c r="I33" s="40" t="s">
-        <v>130</v>
-      </c>
-      <c r="J33" s="41" t="s">
-        <v>131</v>
-      </c>
-      <c r="K33" s="39" t="s">
-        <v>194</v>
       </c>
     </row>
   </sheetData>
@@ -2838,5 +3436,6 @@
     <mergeCell ref="A30:K30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>